<commit_message>
Acrescentei uma forma de ao bipar o QR code o operador vizualizar os dados básicos antes de entrar na planilha
</commit_message>
<xml_diff>
--- a/modelos/Etiqueta de faturamento.xlsx
+++ b/modelos/Etiqueta de faturamento.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/484c53c37b433491/Desktop/Projetos/Transformers - Convertedor de arquivos/modelos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{84BFC2FC-5254-4369-8D70-55DC78B5005B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="169" documentId="8_{84BFC2FC-5254-4369-8D70-55DC78B5005B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B6F3868A-4D1E-47DF-9A4A-9BDA12E4C5F5}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C109A394-F70B-4C9C-9BDE-35484F4354EC}"/>
   </bookViews>
@@ -38,6 +38,28 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
+  <metadataTypes count="1">
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLRICHVALUE" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <valueMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </valueMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
@@ -53,12 +75,12 @@
     <t>Data:</t>
   </si>
   <si>
-    <t>Se possuir alguma solicitação ou sugestão com relação à
-montagem dos pallets, favor enviar e-mail para:
-contato@luariembalagens.com.br</t>
+    <t>www.luariembalagens.com.br</t>
   </si>
   <si>
-    <t>www.luariembalagens.com.br</t>
+    <t>Se possuir alguma solicitação ou sugestão com relação à
+montagem dos pallets, favor enviar na pesquisa de qualidade do QR Code fixado ou um e-mail para:
+contato@luariembalagens.com.br</t>
   </si>
 </sst>
 </file>
@@ -114,7 +136,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -225,56 +247,105 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="3"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -296,25 +367,63 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>585142</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>74543</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1789044" cy="679175"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="image1.png" title="Imagem">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AD9C610E-C020-4430-B66B-A19CF00B05D2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="585142" y="74543"/>
+          <a:ext cx="1789044" cy="679175"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>952499</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>66262</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>863507</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>8400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>1350065</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>182219</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1086531</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>230882</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Imagem 1">
+        <xdr:cNvPr id="8" name="Gráfico 7" descr="Contorno de rosto divertido com preenchimento sólido">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DDBDF759-6F7A-4F86-B0B5-99D076E44C0F}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{901ED223-93F1-44FD-9DC9-CFCDC01E57DA}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -322,23 +431,122 @@
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
           <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId3"/>
             </a:ext>
           </a:extLst>
         </a:blip>
-        <a:srcRect l="15088" t="39298" r="17193" b="31579"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="952499" y="256762"/>
-          <a:ext cx="1597716" cy="687457"/>
+          <a:off x="3149507" y="5521177"/>
+          <a:ext cx="223024" cy="222482"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>452297</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>12255</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>678651</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>238059</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Gráfico 9" descr="Contorno de rosto nervoso com preenchimento sólido">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{85B4D4D5-BB80-0CF7-BAC0-1EB621C83E6D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4">
+          <a:extLst>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId5"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2738297" y="5525032"/>
+          <a:ext cx="226354" cy="225804"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>37160</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>8978</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>257551</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>229369</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="Gráfico 11" descr="Contorno de rosto irritado com preenchimento sólido">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3F728539-C11D-9270-08A9-C2028542B018}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6">
+          <a:extLst>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId7"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2323160" y="5521755"/>
+          <a:ext cx="220391" cy="220391"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -348,6 +556,74 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <rv s="0">
+    <v>0</v>
+    <v>5</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <s t="_localImage">
+    <k n="_rvRel:LocalImageIdentifier" t="i"/>
+    <k n="CalcOrigin" t="i"/>
+  </s>
+</rvStructures>
+</file>
+
+<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
+<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <rel r:id="rId1"/>
+</richValueRels>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -667,136 +943,171 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D18FFF38-996B-4636-8EC2-E1CA3C8BCABA}">
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="40" customWidth="1"/>
+    <col min="1" max="1" width="11.42578125" customWidth="1"/>
+    <col min="2" max="2" width="22.85546875" customWidth="1"/>
+    <col min="3" max="3" width="17.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1"/>
-      <c r="B1" s="2"/>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="3"/>
-      <c r="B2" s="4"/>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="3"/>
-      <c r="B3" s="4"/>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="3"/>
-      <c r="B4" s="4"/>
-    </row>
-    <row r="5" spans="1:2" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="5"/>
-      <c r="B5" s="6"/>
-    </row>
-    <row r="6" spans="1:2" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+    <row r="1" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="9"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+    </row>
+    <row r="2" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="9"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+    </row>
+    <row r="3" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="9"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+    </row>
+    <row r="4" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="9"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+    </row>
+    <row r="5" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="10"/>
+      <c r="C5" s="9"/>
+    </row>
+    <row r="6" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="8"/>
-    </row>
-    <row r="7" spans="1:2" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
+      <c r="B6" s="5"/>
+      <c r="C6" s="6"/>
+    </row>
+    <row r="7" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="8"/>
-    </row>
-    <row r="8" spans="1:2" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
+      <c r="B7" s="5"/>
+      <c r="C7" s="6"/>
+    </row>
+    <row r="8" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="8"/>
-    </row>
-    <row r="9" spans="1:2" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
+      <c r="B8" s="5"/>
+      <c r="C8" s="6"/>
+    </row>
+    <row r="9" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="8"/>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="9"/>
-      <c r="B10" s="10"/>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="10"/>
-      <c r="B11" s="10"/>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="10"/>
-      <c r="B12" s="10"/>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="10"/>
-      <c r="B13" s="10"/>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="10"/>
-      <c r="B14" s="10"/>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="10"/>
-      <c r="B15" s="10"/>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="10"/>
-      <c r="B16" s="10"/>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="10"/>
-      <c r="B17" s="10"/>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="10"/>
-      <c r="B18" s="10"/>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="10"/>
-      <c r="B19" s="10"/>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="10"/>
-      <c r="B20" s="10"/>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="10"/>
-      <c r="B21" s="10"/>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="10"/>
-      <c r="B22" s="10"/>
-    </row>
-    <row r="23" spans="1:2" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="B23" s="12"/>
-    </row>
-    <row r="24" spans="1:2" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="13"/>
-      <c r="B24" s="14"/>
-    </row>
-    <row r="25" spans="1:2" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="15" t="s">
+      <c r="B9" s="5"/>
+      <c r="C9" s="6"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="11"/>
+      <c r="B10" s="12"/>
+      <c r="C10" s="13"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="14"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="16"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="14"/>
+      <c r="B12" s="15"/>
+      <c r="C12" s="16"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="14"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="16"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="14"/>
+      <c r="B14" s="15"/>
+      <c r="C14" s="16"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="14"/>
+      <c r="B15" s="15"/>
+      <c r="C15" s="16"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="14"/>
+      <c r="B16" s="15"/>
+      <c r="C16" s="16"/>
+      <c r="G16" s="3"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="14"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="16"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="14"/>
+      <c r="B18" s="15"/>
+      <c r="C18" s="16"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="14"/>
+      <c r="B19" s="15"/>
+      <c r="C19" s="16"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="14"/>
+      <c r="B20" s="15"/>
+      <c r="C20" s="16"/>
+    </row>
+    <row r="21" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="17"/>
+      <c r="B21" s="18"/>
+      <c r="C21" s="19"/>
+    </row>
+    <row r="22" spans="1:3" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="B25" s="16"/>
+      <c r="B22" s="21"/>
+      <c r="C22" s="7" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="22"/>
+      <c r="B23" s="23"/>
+      <c r="C23" s="8"/>
+    </row>
+    <row r="24" spans="1:3" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="22"/>
+      <c r="B24" s="23"/>
+      <c r="C24" s="8"/>
+    </row>
+    <row r="25" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="24"/>
+      <c r="B25" s="25"/>
+      <c r="C25" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A1:B5"/>
-    <mergeCell ref="A10:B22"/>
-    <mergeCell ref="A23:B24"/>
-    <mergeCell ref="A25:B25"/>
+  <mergeCells count="9">
+    <mergeCell ref="A1:C4"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A10:C21"/>
+    <mergeCell ref="A22:B25"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="C22:C24"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A25" r:id="rId1" xr:uid="{62D512AE-B121-4E9B-B189-32D735EB199D}"/>
+    <hyperlink ref="A5" r:id="rId1" xr:uid="{815B3961-030E-4A96-BC25-E64923DA3D1E}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <drawing r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <drawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>